<commit_message>
#15 Client BOM updated.
</commit_message>
<xml_diff>
--- a/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Client BOM tracker-pro-airbnb-v1.1.xlsx
+++ b/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Client BOM tracker-pro-airbnb-v1.1.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="599">
   <si>
     <t>#</t>
   </si>
@@ -1795,13 +1795,34 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>100% Original 3.7V 18500 2040mah Lithium Ion Battery for Panasonic NCR18500A 3.6V Battery for Toy Torch Flashlight Ect</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Sensor</t>
+  </si>
+  <si>
+    <t>PMS5003</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1865,6 +1886,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1892,7 +1928,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -2023,11 +2059,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2093,9 +2167,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2114,8 +2185,33 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2401,7 +2497,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I135"/>
+  <dimension ref="A1:J137"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" style="6" bestFit="1" customWidth="1"/>
@@ -2412,10 +2508,11 @@
     <col min="6" max="6" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.42578125" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4"/>
       <c r="B1" s="4"/>
       <c r="C1" s="1"/>
@@ -2423,10 +2520,11 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
@@ -2452,15 +2550,18 @@
         <v>590</v>
       </c>
       <c r="I2" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="J2" s="29" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20">
         <f>ROW(A3) - ROW($A$2)</f>
         <v>1</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="14" t="s">
@@ -2481,16 +2582,17 @@
       <c r="H3" s="15" t="s">
         <v>529</v>
       </c>
-      <c r="I3" s="14">
+      <c r="I3" s="14"/>
+      <c r="J3" s="30">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="20">
         <f t="shared" ref="A4:A132" si="0">ROW(A4) - ROW($A$2)</f>
         <v>2</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="16" t="s">
@@ -2511,16 +2613,17 @@
       <c r="H4" s="17" t="s">
         <v>530</v>
       </c>
-      <c r="I4" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I4" s="16"/>
+      <c r="J4" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="20">
         <f>ROW(A5) - ROW($A$2)</f>
         <v>3</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="14" t="s">
@@ -2541,16 +2644,17 @@
       <c r="H5" s="15" t="s">
         <v>531</v>
       </c>
-      <c r="I5" s="14">
+      <c r="I5" s="14"/>
+      <c r="J5" s="30">
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="20">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="16" t="s">
@@ -2571,16 +2675,17 @@
       <c r="H6" s="17" t="s">
         <v>532</v>
       </c>
-      <c r="I6" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I6" s="16"/>
+      <c r="J6" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="20">
         <f>ROW(A7) - ROW($A$2)</f>
         <v>5</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="14" t="s">
@@ -2601,16 +2706,17 @@
       <c r="H7" s="15" t="s">
         <v>533</v>
       </c>
-      <c r="I7" s="14">
+      <c r="I7" s="14"/>
+      <c r="J7" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="20">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C8" s="16" t="s">
@@ -2631,16 +2737,17 @@
       <c r="H8" s="17" t="s">
         <v>534</v>
       </c>
-      <c r="I8" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I8" s="16"/>
+      <c r="J8" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="20">
         <f>ROW(A9) - ROW($A$2)</f>
         <v>7</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="14" t="s">
@@ -2661,16 +2768,17 @@
       <c r="H9" s="15" t="s">
         <v>535</v>
       </c>
-      <c r="I9" s="14">
+      <c r="I9" s="14"/>
+      <c r="J9" s="30">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="20">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C10" s="16" t="s">
@@ -2691,16 +2799,17 @@
       <c r="H10" s="17" t="s">
         <v>536</v>
       </c>
-      <c r="I10" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I10" s="16"/>
+      <c r="J10" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="20">
         <f>ROW(A11) - ROW($A$2)</f>
         <v>9</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C11" s="14" t="s">
@@ -2721,16 +2830,17 @@
       <c r="H11" s="15" t="s">
         <v>537</v>
       </c>
-      <c r="I11" s="14">
+      <c r="I11" s="14"/>
+      <c r="J11" s="30">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="20">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="16" t="s">
@@ -2751,16 +2861,17 @@
       <c r="H12" s="17" t="s">
         <v>538</v>
       </c>
-      <c r="I12" s="16">
+      <c r="I12" s="16"/>
+      <c r="J12" s="31">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="20">
         <f>ROW(A13) - ROW($A$2)</f>
         <v>11</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C13" s="14" t="s">
@@ -2781,16 +2892,17 @@
       <c r="H13" s="15" t="s">
         <v>539</v>
       </c>
-      <c r="I13" s="14">
+      <c r="I13" s="14"/>
+      <c r="J13" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="20">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C14" s="16" t="s">
@@ -2811,16 +2923,17 @@
       <c r="H14" s="17" t="s">
         <v>529</v>
       </c>
-      <c r="I14" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I14" s="16"/>
+      <c r="J14" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="20">
         <f>ROW(A15) - ROW($A$2)</f>
         <v>13</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -2841,16 +2954,17 @@
       <c r="H15" s="15" t="s">
         <v>540</v>
       </c>
-      <c r="I15" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I15" s="14"/>
+      <c r="J15" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="20">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C16" s="16" t="s">
@@ -2871,16 +2985,17 @@
       <c r="H16" s="17" t="s">
         <v>541</v>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="16"/>
+      <c r="J16" s="31">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="20">
         <f>ROW(A17) - ROW($A$2)</f>
         <v>15</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C17" s="14" t="s">
@@ -2901,16 +3016,17 @@
       <c r="H17" s="15" t="s">
         <v>533</v>
       </c>
-      <c r="I17" s="14">
+      <c r="I17" s="14"/>
+      <c r="J17" s="30">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="20">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C18" s="16" t="s">
@@ -2931,16 +3047,17 @@
       <c r="H18" s="17" t="s">
         <v>542</v>
       </c>
-      <c r="I18" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I18" s="16"/>
+      <c r="J18" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="20">
         <f>ROW(A19) - ROW($A$2)</f>
         <v>17</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C19" s="14" t="s">
@@ -2961,16 +3078,17 @@
       <c r="H19" s="15" t="s">
         <v>531</v>
       </c>
-      <c r="I19" s="14">
+      <c r="I19" s="14"/>
+      <c r="J19" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="20">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C20" s="16" t="s">
@@ -2991,16 +3109,17 @@
       <c r="H20" s="17" t="s">
         <v>543</v>
       </c>
-      <c r="I20" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I20" s="16"/>
+      <c r="J20" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="20">
         <f>ROW(A21) - ROW($A$2)</f>
         <v>19</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C21" s="14" t="s">
@@ -3021,16 +3140,17 @@
       <c r="H21" s="15" t="s">
         <v>544</v>
       </c>
-      <c r="I21" s="14">
+      <c r="I21" s="14"/>
+      <c r="J21" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="20">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C22" s="16" t="s">
@@ -3051,16 +3171,17 @@
       <c r="H22" s="17" t="s">
         <v>545</v>
       </c>
-      <c r="I22" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I22" s="16"/>
+      <c r="J22" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="20">
         <f>ROW(A23) - ROW($A$2)</f>
         <v>21</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C23" s="14" t="s">
@@ -3081,16 +3202,17 @@
       <c r="H23" s="15" t="s">
         <v>533</v>
       </c>
-      <c r="I23" s="14">
+      <c r="I23" s="14"/>
+      <c r="J23" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="20">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C24" s="16" t="s">
@@ -3111,16 +3233,17 @@
       <c r="H24" s="17" t="s">
         <v>529</v>
       </c>
-      <c r="I24" s="16">
+      <c r="I24" s="16"/>
+      <c r="J24" s="31">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20">
         <f>ROW(A25) - ROW($A$2)</f>
         <v>23</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C25" s="14" t="s">
@@ -3141,16 +3264,17 @@
       <c r="H25" s="15" t="s">
         <v>546</v>
       </c>
-      <c r="I25" s="14">
+      <c r="I25" s="14"/>
+      <c r="J25" s="30">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="20">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C26" s="16" t="s">
@@ -3171,16 +3295,17 @@
       <c r="H26" s="17" t="s">
         <v>547</v>
       </c>
-      <c r="I26" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I26" s="16"/>
+      <c r="J26" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="20">
         <f>ROW(A27) - ROW($A$2)</f>
         <v>25</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C27" s="14" t="s">
@@ -3201,16 +3326,17 @@
       <c r="H27" s="15" t="s">
         <v>548</v>
       </c>
-      <c r="I27" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I27" s="14"/>
+      <c r="J27" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="20">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C28" s="16" t="s">
@@ -3231,16 +3357,17 @@
       <c r="H28" s="17" t="s">
         <v>531</v>
       </c>
-      <c r="I28" s="16">
+      <c r="I28" s="16"/>
+      <c r="J28" s="31">
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="20">
         <f>ROW(A29) - ROW($A$2)</f>
         <v>27</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C29" s="14" t="s">
@@ -3261,16 +3388,17 @@
       <c r="H29" s="15" t="s">
         <v>537</v>
       </c>
-      <c r="I29" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I29" s="14"/>
+      <c r="J29" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="20">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C30" s="16" t="s">
@@ -3291,16 +3419,17 @@
       <c r="H30" s="17" t="s">
         <v>549</v>
       </c>
-      <c r="I30" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I30" s="16"/>
+      <c r="J30" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="20">
         <f>ROW(A31) - ROW($A$2)</f>
         <v>29</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C31" s="14" t="s">
@@ -3321,16 +3450,17 @@
       <c r="H31" s="15" t="s">
         <v>531</v>
       </c>
-      <c r="I31" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I31" s="14"/>
+      <c r="J31" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="20">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="21" t="s">
         <v>2</v>
       </c>
       <c r="C32" s="16" t="s">
@@ -3351,16 +3481,17 @@
       <c r="H32" s="17" t="s">
         <v>529</v>
       </c>
-      <c r="I32" s="16">
+      <c r="I32" s="16"/>
+      <c r="J32" s="31">
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="20">
         <f>ROW(A33) - ROW($A$2)</f>
         <v>31</v>
       </c>
-      <c r="B33" s="23" t="s">
+      <c r="B33" s="22" t="s">
         <v>3</v>
       </c>
       <c r="C33" s="14" t="s">
@@ -3381,46 +3512,48 @@
       <c r="H33" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I33" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I33" s="14"/>
+      <c r="J33" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="20">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="C34" s="24" t="s">
+      <c r="C34" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="D34" s="25" t="s">
+      <c r="D34" s="24" t="s">
         <v>198</v>
       </c>
-      <c r="E34" s="24" t="s">
+      <c r="E34" s="23" t="s">
         <v>304</v>
       </c>
-      <c r="F34" s="25" t="s">
+      <c r="F34" s="24" t="s">
         <v>398</v>
       </c>
-      <c r="G34" s="24" t="s">
+      <c r="G34" s="23" t="s">
         <v>485</v>
       </c>
-      <c r="H34" s="25" t="s">
+      <c r="H34" s="24" t="s">
         <v>550</v>
       </c>
-      <c r="I34" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I34" s="23"/>
+      <c r="J34" s="32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="20">
         <f>ROW(A35) - ROW($A$2)</f>
         <v>33</v>
       </c>
-      <c r="B35" s="22" t="s">
+      <c r="B35" s="21" t="s">
         <v>3</v>
       </c>
       <c r="C35" s="14" t="s">
@@ -3441,16 +3574,17 @@
       <c r="H35" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I35" s="14">
+      <c r="I35" s="14"/>
+      <c r="J35" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="20">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="B36" s="23" t="s">
+      <c r="B36" s="22" t="s">
         <v>3</v>
       </c>
       <c r="C36" s="16" t="s">
@@ -3471,16 +3605,17 @@
       <c r="H36" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I36" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I36" s="14"/>
+      <c r="J36" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="20">
         <f>ROW(A37) - ROW($A$2)</f>
         <v>35</v>
       </c>
-      <c r="B37" s="22" t="s">
+      <c r="B37" s="21" t="s">
         <v>3</v>
       </c>
       <c r="C37" s="14" t="s">
@@ -3501,16 +3636,17 @@
       <c r="H37" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I37" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I37" s="14"/>
+      <c r="J37" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="20">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="B38" s="23" t="s">
+      <c r="B38" s="22" t="s">
         <v>3</v>
       </c>
       <c r="C38" s="16" t="s">
@@ -3531,16 +3667,17 @@
       <c r="H38" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I38" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I38" s="14"/>
+      <c r="J38" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="20">
         <f>ROW(A39) - ROW($A$2)</f>
         <v>37</v>
       </c>
-      <c r="B39" s="22" t="s">
+      <c r="B39" s="21" t="s">
         <v>3</v>
       </c>
       <c r="C39" s="14" t="s">
@@ -3561,16 +3698,17 @@
       <c r="H39" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I39" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I39" s="14"/>
+      <c r="J39" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="20">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="B40" s="23" t="s">
+      <c r="B40" s="22" t="s">
         <v>4</v>
       </c>
       <c r="C40" s="16" t="s">
@@ -3591,16 +3729,17 @@
       <c r="H40" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I40" s="16">
+      <c r="I40" s="14"/>
+      <c r="J40" s="31">
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="20">
         <f>ROW(A41) - ROW($A$2)</f>
         <v>39</v>
       </c>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="21" t="s">
         <v>5</v>
       </c>
       <c r="C41" s="14" t="s">
@@ -3621,16 +3760,17 @@
       <c r="H41" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I41" s="14">
+      <c r="I41" s="14"/>
+      <c r="J41" s="30">
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="20">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="B42" s="23" t="s">
+      <c r="B42" s="22" t="s">
         <v>5</v>
       </c>
       <c r="C42" s="16" t="s">
@@ -3651,16 +3791,17 @@
       <c r="H42" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I42" s="16">
+      <c r="I42" s="14"/>
+      <c r="J42" s="31">
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="20">
         <f>ROW(A43) - ROW($A$2)</f>
         <v>41</v>
       </c>
-      <c r="B43" s="22" t="s">
+      <c r="B43" s="21" t="s">
         <v>5</v>
       </c>
       <c r="C43" s="14" t="s">
@@ -3681,16 +3822,17 @@
       <c r="H43" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I43" s="14">
+      <c r="I43" s="14"/>
+      <c r="J43" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="20">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="B44" s="23" t="s">
+      <c r="B44" s="22" t="s">
         <v>5</v>
       </c>
       <c r="C44" s="16" t="s">
@@ -3711,16 +3853,17 @@
       <c r="H44" s="17" t="s">
         <v>551</v>
       </c>
-      <c r="I44" s="16">
+      <c r="I44" s="16"/>
+      <c r="J44" s="31">
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="20">
         <f>ROW(A45) - ROW($A$2)</f>
         <v>43</v>
       </c>
-      <c r="B45" s="22" t="s">
+      <c r="B45" s="21" t="s">
         <v>6</v>
       </c>
       <c r="C45" s="14" t="s">
@@ -3741,16 +3884,17 @@
       <c r="H45" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I45" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I45" s="14"/>
+      <c r="J45" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="20">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="B46" s="23" t="s">
+      <c r="B46" s="22" t="s">
         <v>7</v>
       </c>
       <c r="C46" s="16" t="s">
@@ -3771,16 +3915,17 @@
       <c r="H46" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I46" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I46" s="14"/>
+      <c r="J46" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="20">
         <f>ROW(A47) - ROW($A$2)</f>
         <v>45</v>
       </c>
-      <c r="B47" s="22" t="s">
+      <c r="B47" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C47" s="14" t="s">
@@ -3801,16 +3946,17 @@
       <c r="H47" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I47" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I47" s="14"/>
+      <c r="J47" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="20">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="B48" s="23" t="s">
+      <c r="B48" s="22" t="s">
         <v>9</v>
       </c>
       <c r="C48" s="16" t="s">
@@ -3831,16 +3977,17 @@
       <c r="H48" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I48" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I48" s="14"/>
+      <c r="J48" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="20">
         <f>ROW(A49) - ROW($A$2)</f>
         <v>47</v>
       </c>
-      <c r="B49" s="22" t="s">
+      <c r="B49" s="21" t="s">
         <v>10</v>
       </c>
       <c r="C49" s="14" t="s">
@@ -3861,16 +4008,17 @@
       <c r="H49" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I49" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I49" s="14"/>
+      <c r="J49" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="20">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="B50" s="23" t="s">
+      <c r="B50" s="22" t="s">
         <v>11</v>
       </c>
       <c r="C50" s="16" t="s">
@@ -3891,16 +4039,17 @@
       <c r="H50" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I50" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I50" s="14"/>
+      <c r="J50" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="20">
         <f>ROW(A51) - ROW($A$2)</f>
         <v>49</v>
       </c>
-      <c r="B51" s="22" t="s">
+      <c r="B51" s="21" t="s">
         <v>12</v>
       </c>
       <c r="C51" s="14" t="s">
@@ -3921,16 +4070,17 @@
       <c r="H51" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I51" s="14">
+      <c r="I51" s="14"/>
+      <c r="J51" s="30">
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="20">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="B52" s="23" t="s">
+      <c r="B52" s="22" t="s">
         <v>13</v>
       </c>
       <c r="C52" s="16" t="s">
@@ -3949,16 +4099,17 @@
       <c r="H52" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I52" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I52" s="14"/>
+      <c r="J52" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="20">
         <f>ROW(A53) - ROW($A$2)</f>
         <v>51</v>
       </c>
-      <c r="B53" s="22" t="s">
+      <c r="B53" s="21" t="s">
         <v>14</v>
       </c>
       <c r="C53" s="14" t="s">
@@ -3979,16 +4130,17 @@
       <c r="H53" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I53" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I53" s="14"/>
+      <c r="J53" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="20">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="B54" s="23" t="s">
+      <c r="B54" s="22" t="s">
         <v>15</v>
       </c>
       <c r="C54" s="16" t="s">
@@ -4009,16 +4161,17 @@
       <c r="H54" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I54" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I54" s="14"/>
+      <c r="J54" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="20">
         <f>ROW(A55) - ROW($A$2)</f>
         <v>53</v>
       </c>
-      <c r="B55" s="22" t="s">
+      <c r="B55" s="21" t="s">
         <v>16</v>
       </c>
       <c r="C55" s="14" t="s">
@@ -4039,16 +4192,17 @@
       <c r="H55" s="15" t="s">
         <v>552</v>
       </c>
-      <c r="I55" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I55" s="14"/>
+      <c r="J55" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="20">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="B56" s="23" t="s">
+      <c r="B56" s="22" t="s">
         <v>16</v>
       </c>
       <c r="C56" s="16" t="s">
@@ -4069,16 +4223,17 @@
       <c r="H56" s="17" t="s">
         <v>553</v>
       </c>
-      <c r="I56" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I56" s="16"/>
+      <c r="J56" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="20">
         <f>ROW(A57) - ROW($A$2)</f>
         <v>55</v>
       </c>
-      <c r="B57" s="22" t="s">
+      <c r="B57" s="21" t="s">
         <v>16</v>
       </c>
       <c r="C57" s="14" t="s">
@@ -4099,16 +4254,17 @@
       <c r="H57" s="15" t="s">
         <v>554</v>
       </c>
-      <c r="I57" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I57" s="14"/>
+      <c r="J57" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="20">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="B58" s="23" t="s">
+      <c r="B58" s="22" t="s">
         <v>16</v>
       </c>
       <c r="C58" s="16" t="s">
@@ -4129,16 +4285,17 @@
       <c r="H58" s="17" t="s">
         <v>555</v>
       </c>
-      <c r="I58" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I58" s="16"/>
+      <c r="J58" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="20">
         <f>ROW(A59) - ROW($A$2)</f>
         <v>57</v>
       </c>
-      <c r="B59" s="22" t="s">
+      <c r="B59" s="21" t="s">
         <v>17</v>
       </c>
       <c r="C59" s="14" t="s">
@@ -4159,16 +4316,17 @@
       <c r="H59" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I59" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I59" s="14"/>
+      <c r="J59" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="20">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="B60" s="23" t="s">
+      <c r="B60" s="22" t="s">
         <v>17</v>
       </c>
       <c r="C60" s="16" t="s">
@@ -4189,16 +4347,17 @@
       <c r="H60" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I60" s="16">
+      <c r="I60" s="14"/>
+      <c r="J60" s="31">
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="20">
         <f>ROW(A61) - ROW($A$2)</f>
         <v>59</v>
       </c>
-      <c r="B61" s="22" t="s">
+      <c r="B61" s="21" t="s">
         <v>17</v>
       </c>
       <c r="C61" s="14" t="s">
@@ -4219,16 +4378,17 @@
       <c r="H61" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I61" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I61" s="14"/>
+      <c r="J61" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="20">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="B62" s="23" t="s">
+      <c r="B62" s="22" t="s">
         <v>18</v>
       </c>
       <c r="C62" s="16" t="s">
@@ -4249,72 +4409,75 @@
       <c r="H62" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I62" s="16">
+      <c r="I62" s="14"/>
+      <c r="J62" s="31">
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="20">
         <f>ROW(A63) - ROW($A$2)</f>
         <v>61</v>
       </c>
-      <c r="B63" s="22" t="s">
+      <c r="B63" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C63" s="26" t="s">
+      <c r="C63" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="D63" s="27" t="s">
+      <c r="D63" s="26" t="s">
         <v>225</v>
       </c>
-      <c r="E63" s="26" t="s">
+      <c r="E63" s="25" t="s">
         <v>329</v>
       </c>
-      <c r="F63" s="27"/>
-      <c r="G63" s="26"/>
-      <c r="H63" s="27" t="s">
+      <c r="F63" s="26"/>
+      <c r="G63" s="25"/>
+      <c r="H63" s="26" t="s">
         <v>591</v>
       </c>
-      <c r="I63" s="26">
+      <c r="I63" s="25"/>
+      <c r="J63" s="33">
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="20">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="B64" s="23" t="s">
+      <c r="B64" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C64" s="24" t="s">
+      <c r="C64" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="D64" s="25" t="s">
+      <c r="D64" s="24" t="s">
         <v>226</v>
       </c>
-      <c r="E64" s="24" t="s">
+      <c r="E64" s="23" t="s">
         <v>330</v>
       </c>
-      <c r="F64" s="25" t="s">
+      <c r="F64" s="24" t="s">
         <v>416</v>
       </c>
-      <c r="G64" s="24" t="s">
+      <c r="G64" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="H64" s="25" t="s">
+      <c r="H64" s="24" t="s">
         <v>550</v>
       </c>
-      <c r="I64" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I64" s="23"/>
+      <c r="J64" s="32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="20">
         <f>ROW(A65) - ROW($A$2)</f>
         <v>63</v>
       </c>
-      <c r="B65" s="22" t="s">
+      <c r="B65" s="21" t="s">
         <v>20</v>
       </c>
       <c r="C65" s="14" t="s">
@@ -4335,16 +4498,17 @@
       <c r="H65" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I65" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I65" s="14"/>
+      <c r="J65" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="20">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
-      <c r="B66" s="23" t="s">
+      <c r="B66" s="22" t="s">
         <v>20</v>
       </c>
       <c r="C66" s="16" t="s">
@@ -4365,16 +4529,17 @@
       <c r="H66" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I66" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I66" s="14"/>
+      <c r="J66" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="20">
         <f>ROW(A67) - ROW($A$2)</f>
         <v>65</v>
       </c>
-      <c r="B67" s="22" t="s">
+      <c r="B67" s="21" t="s">
         <v>20</v>
       </c>
       <c r="C67" s="14" t="s">
@@ -4395,16 +4560,17 @@
       <c r="H67" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I67" s="14">
+      <c r="I67" s="14"/>
+      <c r="J67" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="20">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="B68" s="23" t="s">
+      <c r="B68" s="22" t="s">
         <v>20</v>
       </c>
       <c r="C68" s="16" t="s">
@@ -4425,16 +4591,17 @@
       <c r="H68" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I68" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I68" s="14"/>
+      <c r="J68" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="20">
         <f>ROW(A69) - ROW($A$2)</f>
         <v>67</v>
       </c>
-      <c r="B69" s="22" t="s">
+      <c r="B69" s="21" t="s">
         <v>20</v>
       </c>
       <c r="C69" s="14" t="s">
@@ -4455,16 +4622,17 @@
       <c r="H69" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I69" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I69" s="14"/>
+      <c r="J69" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="20">
         <f t="shared" si="0"/>
         <v>68</v>
       </c>
-      <c r="B70" s="22" t="s">
+      <c r="B70" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C70" s="16" t="s">
@@ -4485,16 +4653,17 @@
       <c r="H70" s="17" t="s">
         <v>556</v>
       </c>
-      <c r="I70" s="16">
+      <c r="I70" s="16"/>
+      <c r="J70" s="31">
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="20">
         <f>ROW(A71) - ROW($A$2)</f>
         <v>69</v>
       </c>
-      <c r="B71" s="22" t="s">
+      <c r="B71" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C71" s="14" t="s">
@@ -4515,16 +4684,17 @@
       <c r="H71" s="15" t="s">
         <v>557</v>
       </c>
-      <c r="I71" s="14">
+      <c r="I71" s="14"/>
+      <c r="J71" s="30">
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="20">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="B72" s="23" t="s">
+      <c r="B72" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C72" s="16" t="s">
@@ -4545,16 +4715,17 @@
       <c r="H72" s="17" t="s">
         <v>558</v>
       </c>
-      <c r="I72" s="16">
+      <c r="I72" s="16"/>
+      <c r="J72" s="31">
         <v>20</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="20">
         <f>ROW(A73) - ROW($A$2)</f>
         <v>71</v>
       </c>
-      <c r="B73" s="22" t="s">
+      <c r="B73" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C73" s="14" t="s">
@@ -4575,16 +4746,17 @@
       <c r="H73" s="15" t="s">
         <v>559</v>
       </c>
-      <c r="I73" s="14">
+      <c r="I73" s="14"/>
+      <c r="J73" s="30">
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="20">
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="B74" s="23" t="s">
+      <c r="B74" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C74" s="16" t="s">
@@ -4605,16 +4777,17 @@
       <c r="H74" s="17" t="s">
         <v>560</v>
       </c>
-      <c r="I74" s="16">
+      <c r="I74" s="16"/>
+      <c r="J74" s="31">
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="20">
         <f>ROW(A75) - ROW($A$2)</f>
         <v>73</v>
       </c>
-      <c r="B75" s="23" t="s">
+      <c r="B75" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C75" s="14" t="s">
@@ -4635,16 +4808,17 @@
       <c r="H75" s="15" t="s">
         <v>561</v>
       </c>
-      <c r="I75" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I75" s="14"/>
+      <c r="J75" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="20">
         <f t="shared" si="0"/>
         <v>74</v>
       </c>
-      <c r="B76" s="23" t="s">
+      <c r="B76" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C76" s="16" t="s">
@@ -4665,16 +4839,17 @@
       <c r="H76" s="17" t="s">
         <v>562</v>
       </c>
-      <c r="I76" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I76" s="16"/>
+      <c r="J76" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="20">
         <f>ROW(A77) - ROW($A$2)</f>
         <v>75</v>
       </c>
-      <c r="B77" s="22" t="s">
+      <c r="B77" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C77" s="14" t="s">
@@ -4695,16 +4870,17 @@
       <c r="H77" s="15" t="s">
         <v>563</v>
       </c>
-      <c r="I77" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I77" s="14"/>
+      <c r="J77" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="20">
         <f t="shared" si="0"/>
         <v>76</v>
       </c>
-      <c r="B78" s="23" t="s">
+      <c r="B78" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C78" s="16" t="s">
@@ -4725,46 +4901,48 @@
       <c r="H78" s="17" t="s">
         <v>564</v>
       </c>
-      <c r="I78" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I78" s="16"/>
+      <c r="J78" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="20">
         <f>ROW(A79) - ROW($A$2)</f>
         <v>77</v>
       </c>
-      <c r="B79" s="22" t="s">
+      <c r="B79" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C79" s="26" t="s">
+      <c r="C79" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="D79" s="27" t="s">
+      <c r="D79" s="26" t="s">
         <v>240</v>
       </c>
-      <c r="E79" s="26" t="s">
+      <c r="E79" s="25" t="s">
         <v>332</v>
       </c>
-      <c r="F79" s="27" t="s">
+      <c r="F79" s="26" t="s">
         <v>430</v>
       </c>
-      <c r="G79" s="26" t="s">
+      <c r="G79" s="25" t="s">
         <v>475</v>
       </c>
-      <c r="H79" s="27" t="s">
+      <c r="H79" s="26" t="s">
         <v>550</v>
       </c>
-      <c r="I79" s="26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I79" s="25"/>
+      <c r="J79" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="20">
         <f t="shared" si="0"/>
         <v>78</v>
       </c>
-      <c r="B80" s="23" t="s">
+      <c r="B80" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C80" s="16" t="s">
@@ -4785,16 +4963,17 @@
       <c r="H80" s="17" t="s">
         <v>565</v>
       </c>
-      <c r="I80" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I80" s="16"/>
+      <c r="J80" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="20">
         <f>ROW(A81) - ROW($A$2)</f>
         <v>79</v>
       </c>
-      <c r="B81" s="22" t="s">
+      <c r="B81" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C81" s="14" t="s">
@@ -4815,16 +4994,17 @@
       <c r="H81" s="15" t="s">
         <v>566</v>
       </c>
-      <c r="I81" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I81" s="14"/>
+      <c r="J81" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="20">
         <f t="shared" si="0"/>
         <v>80</v>
       </c>
-      <c r="B82" s="23" t="s">
+      <c r="B82" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C82" s="16" t="s">
@@ -4845,16 +5025,17 @@
       <c r="H82" s="17" t="s">
         <v>567</v>
       </c>
-      <c r="I82" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I82" s="16"/>
+      <c r="J82" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="20">
         <f>ROW(A83) - ROW($A$2)</f>
         <v>81</v>
       </c>
-      <c r="B83" s="22" t="s">
+      <c r="B83" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C83" s="14" t="s">
@@ -4875,16 +5056,17 @@
       <c r="H83" s="15" t="s">
         <v>568</v>
       </c>
-      <c r="I83" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I83" s="14"/>
+      <c r="J83" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="20">
         <f t="shared" si="0"/>
         <v>82</v>
       </c>
-      <c r="B84" s="22" t="s">
+      <c r="B84" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C84" s="16" t="s">
@@ -4905,16 +5087,17 @@
       <c r="H84" s="17" t="s">
         <v>569</v>
       </c>
-      <c r="I84" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="85" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I84" s="16"/>
+      <c r="J84" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="20">
         <f>ROW(A85) - ROW($A$2)</f>
         <v>83</v>
       </c>
-      <c r="B85" s="22" t="s">
+      <c r="B85" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C85" s="14" t="s">
@@ -4935,16 +5118,17 @@
       <c r="H85" s="15" t="s">
         <v>558</v>
       </c>
-      <c r="I85" s="14">
+      <c r="I85" s="14"/>
+      <c r="J85" s="30">
         <v>6</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="20">
         <f t="shared" si="0"/>
         <v>84</v>
       </c>
-      <c r="B86" s="23" t="s">
+      <c r="B86" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C86" s="16" t="s">
@@ -4965,16 +5149,17 @@
       <c r="H86" s="17" t="s">
         <v>570</v>
       </c>
-      <c r="I86" s="16">
+      <c r="I86" s="16"/>
+      <c r="J86" s="31">
         <v>3</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="20">
         <f>ROW(A87) - ROW($A$2)</f>
         <v>85</v>
       </c>
-      <c r="B87" s="22" t="s">
+      <c r="B87" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C87" s="14" t="s">
@@ -4995,16 +5180,17 @@
       <c r="H87" s="15" t="s">
         <v>571</v>
       </c>
-      <c r="I87" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I87" s="14"/>
+      <c r="J87" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="20">
         <f t="shared" si="0"/>
         <v>86</v>
       </c>
-      <c r="B88" s="22" t="s">
+      <c r="B88" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C88" s="16" t="s">
@@ -5025,16 +5211,17 @@
       <c r="H88" s="17" t="s">
         <v>572</v>
       </c>
-      <c r="I88" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I88" s="16"/>
+      <c r="J88" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="20">
         <f>ROW(A89) - ROW($A$2)</f>
         <v>87</v>
       </c>
-      <c r="B89" s="22" t="s">
+      <c r="B89" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C89" s="14" t="s">
@@ -5055,16 +5242,17 @@
       <c r="H89" s="15" t="s">
         <v>573</v>
       </c>
-      <c r="I89" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I89" s="14"/>
+      <c r="J89" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="20">
         <f t="shared" si="0"/>
         <v>88</v>
       </c>
-      <c r="B90" s="23" t="s">
+      <c r="B90" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C90" s="16" t="s">
@@ -5085,16 +5273,17 @@
       <c r="H90" s="17" t="s">
         <v>574</v>
       </c>
-      <c r="I90" s="16">
+      <c r="I90" s="16"/>
+      <c r="J90" s="31">
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="20">
         <f>ROW(A91) - ROW($A$2)</f>
         <v>89</v>
       </c>
-      <c r="B91" s="22" t="s">
+      <c r="B91" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C91" s="14" t="s">
@@ -5115,16 +5304,17 @@
       <c r="H91" s="15" t="s">
         <v>575</v>
       </c>
-      <c r="I91" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I91" s="14"/>
+      <c r="J91" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="20">
         <f t="shared" si="0"/>
         <v>90</v>
       </c>
-      <c r="B92" s="23" t="s">
+      <c r="B92" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C92" s="16" t="s">
@@ -5145,16 +5335,17 @@
       <c r="H92" s="17" t="s">
         <v>576</v>
       </c>
-      <c r="I92" s="16">
+      <c r="I92" s="16"/>
+      <c r="J92" s="31">
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="20">
         <f>ROW(A93) - ROW($A$2)</f>
         <v>91</v>
       </c>
-      <c r="B93" s="22" t="s">
+      <c r="B93" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C93" s="14" t="s">
@@ -5175,16 +5366,17 @@
       <c r="H93" s="15" t="s">
         <v>577</v>
       </c>
-      <c r="I93" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I93" s="14"/>
+      <c r="J93" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="20">
         <f t="shared" si="0"/>
         <v>92</v>
       </c>
-      <c r="B94" s="23" t="s">
+      <c r="B94" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C94" s="16" t="s">
@@ -5205,16 +5397,17 @@
       <c r="H94" s="17" t="s">
         <v>578</v>
       </c>
-      <c r="I94" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I94" s="16"/>
+      <c r="J94" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="20">
         <f>ROW(A95) - ROW($A$2)</f>
         <v>93</v>
       </c>
-      <c r="B95" s="22" t="s">
+      <c r="B95" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C95" s="14" t="s">
@@ -5235,16 +5428,17 @@
       <c r="H95" s="15" t="s">
         <v>579</v>
       </c>
-      <c r="I95" s="14">
+      <c r="I95" s="14"/>
+      <c r="J95" s="30">
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="20">
         <f t="shared" si="0"/>
         <v>94</v>
       </c>
-      <c r="B96" s="23" t="s">
+      <c r="B96" s="22" t="s">
         <v>21</v>
       </c>
       <c r="C96" s="16" t="s">
@@ -5265,16 +5459,17 @@
       <c r="H96" s="17" t="s">
         <v>580</v>
       </c>
-      <c r="I96" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I96" s="16"/>
+      <c r="J96" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="20">
         <f>ROW(A97) - ROW($A$2)</f>
         <v>95</v>
       </c>
-      <c r="B97" s="22" t="s">
+      <c r="B97" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C97" s="14" t="s">
@@ -5295,16 +5490,17 @@
       <c r="H97" s="15" t="s">
         <v>581</v>
       </c>
-      <c r="I97" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I97" s="14"/>
+      <c r="J97" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="20">
         <f t="shared" si="0"/>
         <v>96</v>
       </c>
-      <c r="B98" s="22" t="s">
+      <c r="B98" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C98" s="16" t="s">
@@ -5325,16 +5521,17 @@
       <c r="H98" s="17" t="s">
         <v>582</v>
       </c>
-      <c r="I98" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I98" s="16"/>
+      <c r="J98" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="20">
         <f>ROW(A99) - ROW($A$2)</f>
         <v>97</v>
       </c>
-      <c r="B99" s="22" t="s">
+      <c r="B99" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C99" s="14" t="s">
@@ -5355,16 +5552,17 @@
       <c r="H99" s="15" t="s">
         <v>583</v>
       </c>
-      <c r="I99" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I99" s="14"/>
+      <c r="J99" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="20">
         <f t="shared" si="0"/>
         <v>98</v>
       </c>
-      <c r="B100" s="23" t="s">
+      <c r="B100" s="22" t="s">
         <v>22</v>
       </c>
       <c r="C100" s="16" t="s">
@@ -5385,72 +5583,75 @@
       <c r="H100" s="17" t="s">
         <v>558</v>
       </c>
-      <c r="I100" s="16">
+      <c r="I100" s="16"/>
+      <c r="J100" s="31">
         <v>3</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="20">
         <f>ROW(A101) - ROW($A$2)</f>
         <v>99</v>
       </c>
-      <c r="B101" s="22" t="s">
+      <c r="B101" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C101" s="26" t="s">
+      <c r="C101" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="D101" s="27" t="s">
+      <c r="D101" s="26" t="s">
         <v>261</v>
       </c>
-      <c r="E101" s="26" t="s">
+      <c r="E101" s="25" t="s">
         <v>336</v>
       </c>
-      <c r="F101" s="27" t="s">
+      <c r="F101" s="26" t="s">
         <v>336</v>
       </c>
-      <c r="G101" s="26"/>
-      <c r="H101" s="27" t="s">
+      <c r="G101" s="25"/>
+      <c r="H101" s="26" t="s">
         <v>591</v>
       </c>
-      <c r="I101" s="26">
+      <c r="I101" s="25"/>
+      <c r="J101" s="33">
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="20">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="B102" s="23" t="s">
+      <c r="B102" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C102" s="24" t="s">
+      <c r="C102" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="D102" s="25" t="s">
+      <c r="D102" s="24" t="s">
         <v>261</v>
       </c>
-      <c r="E102" s="24" t="s">
+      <c r="E102" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="F102" s="25" t="s">
+      <c r="F102" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="G102" s="24"/>
-      <c r="H102" s="27" t="s">
+      <c r="G102" s="23"/>
+      <c r="H102" s="26" t="s">
         <v>591</v>
       </c>
-      <c r="I102" s="24">
+      <c r="I102" s="25"/>
+      <c r="J102" s="32">
         <v>2</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="20">
         <f>ROW(A103) - ROW($A$2)</f>
         <v>101</v>
       </c>
-      <c r="B103" s="23" t="s">
+      <c r="B103" s="22" t="s">
         <v>24</v>
       </c>
       <c r="C103" s="14" t="s">
@@ -5471,16 +5672,17 @@
       <c r="H103" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I103" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="104" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I103" s="14"/>
+      <c r="J103" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="20">
         <f t="shared" si="0"/>
         <v>102</v>
       </c>
-      <c r="B104" s="23" t="s">
+      <c r="B104" s="22" t="s">
         <v>24</v>
       </c>
       <c r="C104" s="16" t="s">
@@ -5501,16 +5703,17 @@
       <c r="H104" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I104" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="105" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I104" s="14"/>
+      <c r="J104" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="20">
         <f>ROW(A105) - ROW($A$2)</f>
         <v>103</v>
       </c>
-      <c r="B105" s="22" t="s">
+      <c r="B105" s="21" t="s">
         <v>25</v>
       </c>
       <c r="C105" s="14" t="s">
@@ -5531,16 +5734,17 @@
       <c r="H105" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I105" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="106" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I105" s="14"/>
+      <c r="J105" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A106" s="20">
         <f t="shared" si="0"/>
         <v>104</v>
       </c>
-      <c r="B106" s="23" t="s">
+      <c r="B106" s="22" t="s">
         <v>26</v>
       </c>
       <c r="C106" s="16" t="s">
@@ -5561,16 +5765,17 @@
       <c r="H106" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I106" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="107" spans="1:9" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I106" s="14"/>
+      <c r="J106" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="20">
         <f>ROW(A107) - ROW($A$2)</f>
         <v>105</v>
       </c>
-      <c r="B107" s="22" t="s">
+      <c r="B107" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C107" s="14" t="s">
@@ -5591,16 +5796,17 @@
       <c r="H107" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I107" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="108" spans="1:9" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I107" s="14"/>
+      <c r="J107" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="20">
         <f t="shared" si="0"/>
         <v>106</v>
       </c>
-      <c r="B108" s="23" t="s">
+      <c r="B108" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C108" s="16" t="s">
@@ -5621,16 +5827,17 @@
       <c r="H108" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I108" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I108" s="14"/>
+      <c r="J108" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="20">
         <f>ROW(A109) - ROW($A$2)</f>
         <v>107</v>
       </c>
-      <c r="B109" s="22" t="s">
+      <c r="B109" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C109" s="14" t="s">
@@ -5651,16 +5858,17 @@
       <c r="H109" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I109" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="110" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I109" s="14"/>
+      <c r="J109" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="20">
         <f t="shared" si="0"/>
         <v>108</v>
       </c>
-      <c r="B110" s="23" t="s">
+      <c r="B110" s="22" t="s">
         <v>20</v>
       </c>
       <c r="C110" s="16" t="s">
@@ -5681,16 +5889,17 @@
       <c r="H110" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I110" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="111" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I110" s="14"/>
+      <c r="J110" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="20">
         <f>ROW(A111) - ROW($A$2)</f>
         <v>109</v>
       </c>
-      <c r="B111" s="22" t="s">
+      <c r="B111" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C111" s="14" t="s">
@@ -5711,16 +5920,17 @@
       <c r="H111" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I111" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="112" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I111" s="14"/>
+      <c r="J111" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="20">
         <f t="shared" si="0"/>
         <v>110</v>
       </c>
-      <c r="B112" s="23" t="s">
+      <c r="B112" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C112" s="16" t="s">
@@ -5741,16 +5951,17 @@
       <c r="H112" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I112" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="113" spans="1:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I112" s="14"/>
+      <c r="J112" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="20">
         <f>ROW(A113) - ROW($A$2)</f>
         <v>111</v>
       </c>
-      <c r="B113" s="22" t="s">
+      <c r="B113" s="21" t="s">
         <v>28</v>
       </c>
       <c r="C113" s="14" t="s">
@@ -5771,16 +5982,17 @@
       <c r="H113" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I113" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="114" spans="1:9" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I113" s="14"/>
+      <c r="J113" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" s="20">
         <f t="shared" si="0"/>
         <v>112</v>
       </c>
-      <c r="B114" s="23" t="s">
+      <c r="B114" s="22" t="s">
         <v>29</v>
       </c>
       <c r="C114" s="16" t="s">
@@ -5801,16 +6013,17 @@
       <c r="H114" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I114" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="115" spans="1:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I114" s="14"/>
+      <c r="J114" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="20">
         <f>ROW(A115) - ROW($A$2)</f>
         <v>113</v>
       </c>
-      <c r="B115" s="22" t="s">
+      <c r="B115" s="21" t="s">
         <v>30</v>
       </c>
       <c r="C115" s="14" t="s">
@@ -5831,16 +6044,17 @@
       <c r="H115" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I115" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="116" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I115" s="14"/>
+      <c r="J115" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="20">
         <f t="shared" si="0"/>
         <v>114</v>
       </c>
-      <c r="B116" s="23" t="s">
+      <c r="B116" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C116" s="16" t="s">
@@ -5861,16 +6075,17 @@
       <c r="H116" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I116" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="117" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I116" s="14"/>
+      <c r="J116" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="20">
         <f>ROW(A117) - ROW($A$2)</f>
         <v>115</v>
       </c>
-      <c r="B117" s="22" t="s">
+      <c r="B117" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C117" s="14" t="s">
@@ -5891,16 +6106,17 @@
       <c r="H117" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I117" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="118" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I117" s="14"/>
+      <c r="J117" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="20">
         <f t="shared" si="0"/>
         <v>116</v>
       </c>
-      <c r="B118" s="23" t="s">
+      <c r="B118" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C118" s="16" t="s">
@@ -5921,16 +6137,17 @@
       <c r="H118" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I118" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="119" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I118" s="14"/>
+      <c r="J118" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="20">
         <f>ROW(A119) - ROW($A$2)</f>
         <v>117</v>
       </c>
-      <c r="B119" s="22" t="s">
+      <c r="B119" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C119" s="14" t="s">
@@ -5951,16 +6168,17 @@
       <c r="H119" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I119" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="120" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I119" s="14"/>
+      <c r="J119" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="20">
         <f t="shared" si="0"/>
         <v>118</v>
       </c>
-      <c r="B120" s="23" t="s">
+      <c r="B120" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C120" s="16" t="s">
@@ -5981,16 +6199,17 @@
       <c r="H120" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I120" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="121" spans="1:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I120" s="14"/>
+      <c r="J120" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="20">
         <f>ROW(A121) - ROW($A$2)</f>
         <v>119</v>
       </c>
-      <c r="B121" s="22" t="s">
+      <c r="B121" s="21" t="s">
         <v>31</v>
       </c>
       <c r="C121" s="14" t="s">
@@ -6011,16 +6230,17 @@
       <c r="H121" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I121" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="122" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I121" s="14"/>
+      <c r="J121" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="20">
         <f t="shared" si="0"/>
         <v>120</v>
       </c>
-      <c r="B122" s="23" t="s">
+      <c r="B122" s="22" t="s">
         <v>32</v>
       </c>
       <c r="C122" s="16" t="s">
@@ -6041,16 +6261,17 @@
       <c r="H122" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I122" s="16">
+      <c r="I122" s="14"/>
+      <c r="J122" s="31">
         <v>4</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="20">
         <f>ROW(A123) - ROW($A$2)</f>
         <v>121</v>
       </c>
-      <c r="B123" s="22" t="s">
+      <c r="B123" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C123" s="14" t="s">
@@ -6071,16 +6292,17 @@
       <c r="H123" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I123" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="124" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I123" s="14"/>
+      <c r="J123" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A124" s="20">
         <f t="shared" si="0"/>
         <v>122</v>
       </c>
-      <c r="B124" s="23" t="s">
+      <c r="B124" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C124" s="16" t="s">
@@ -6101,16 +6323,17 @@
       <c r="H124" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I124" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="125" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I124" s="14"/>
+      <c r="J124" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" s="20">
         <f>ROW(A125) - ROW($A$2)</f>
         <v>123</v>
       </c>
-      <c r="B125" s="22" t="s">
+      <c r="B125" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C125" s="14" t="s">
@@ -6131,16 +6354,17 @@
       <c r="H125" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I125" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="126" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I125" s="14"/>
+      <c r="J125" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" s="20">
         <f t="shared" si="0"/>
         <v>124</v>
       </c>
-      <c r="B126" s="23" t="s">
+      <c r="B126" s="22" t="s">
         <v>33</v>
       </c>
       <c r="C126" s="16" t="s">
@@ -6161,16 +6385,17 @@
       <c r="H126" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I126" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="127" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I126" s="14"/>
+      <c r="J126" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="20">
         <f>ROW(A127) - ROW($A$2)</f>
         <v>125</v>
       </c>
-      <c r="B127" s="22" t="s">
+      <c r="B127" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C127" s="14" t="s">
@@ -6191,16 +6416,17 @@
       <c r="H127" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I127" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="128" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I127" s="14"/>
+      <c r="J127" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="20">
         <f t="shared" si="0"/>
         <v>126</v>
       </c>
-      <c r="B128" s="23" t="s">
+      <c r="B128" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C128" s="16" t="s">
@@ -6221,16 +6447,17 @@
       <c r="H128" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="I128" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="129" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I128" s="14"/>
+      <c r="J128" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="20">
         <f>ROW(A129) - ROW($A$2)</f>
         <v>127</v>
       </c>
-      <c r="B129" s="22" t="s">
+      <c r="B129" s="21" t="s">
         <v>34</v>
       </c>
       <c r="C129" s="14" t="s">
@@ -6251,16 +6478,17 @@
       <c r="H129" s="15" t="s">
         <v>584</v>
       </c>
-      <c r="I129" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="130" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I129" s="14"/>
+      <c r="J129" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="20">
         <f t="shared" si="0"/>
         <v>128</v>
       </c>
-      <c r="B130" s="23" t="s">
+      <c r="B130" s="22" t="s">
         <v>34</v>
       </c>
       <c r="C130" s="16" t="s">
@@ -6281,16 +6509,17 @@
       <c r="H130" s="17" t="s">
         <v>585</v>
       </c>
-      <c r="I130" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="131" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I130" s="16"/>
+      <c r="J130" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" s="20">
         <f>ROW(A131) - ROW($A$2)</f>
         <v>129</v>
       </c>
-      <c r="B131" s="22" t="s">
+      <c r="B131" s="21" t="s">
         <v>34</v>
       </c>
       <c r="C131" s="14" t="s">
@@ -6311,16 +6540,17 @@
       <c r="H131" s="15" t="s">
         <v>586</v>
       </c>
-      <c r="I131" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="132" spans="1:9" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I131" s="14"/>
+      <c r="J131" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" s="20">
         <f t="shared" si="0"/>
         <v>130</v>
       </c>
-      <c r="B132" s="23" t="s">
+      <c r="B132" s="22" t="s">
         <v>34</v>
       </c>
       <c r="C132" s="16" t="s">
@@ -6341,16 +6571,17 @@
       <c r="H132" s="17" t="s">
         <v>587</v>
       </c>
-      <c r="I132" s="16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="133" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I132" s="16"/>
+      <c r="J132" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="20">
         <f>ROW(A133) - ROW($A$2)</f>
         <v>131</v>
       </c>
-      <c r="B133" s="22" t="s">
+      <c r="B133" s="21" t="s">
         <v>34</v>
       </c>
       <c r="C133" s="14" t="s">
@@ -6371,37 +6602,95 @@
       <c r="H133" s="15" t="s">
         <v>588</v>
       </c>
-      <c r="I133" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A134" s="9"/>
-      <c r="B134" s="18"/>
-      <c r="C134" s="10"/>
-      <c r="D134" s="11"/>
-      <c r="E134" s="12"/>
-      <c r="F134" s="13"/>
-      <c r="G134" s="12"/>
-      <c r="H134" s="13"/>
-      <c r="I134" s="13"/>
-    </row>
-    <row r="135" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="5"/>
-      <c r="B135" s="19"/>
-      <c r="C135" s="2"/>
-      <c r="D135" s="3"/>
-      <c r="E135" s="3"/>
-      <c r="F135" s="3"/>
-      <c r="G135" s="3"/>
-      <c r="H135" s="3"/>
-      <c r="I135" s="3"/>
+      <c r="I133" s="14"/>
+      <c r="J133" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="20">
+        <f t="shared" ref="A134:A135" si="1">ROW(A134) - ROW($A$2)</f>
+        <v>132</v>
+      </c>
+      <c r="B134" s="28" t="s">
+        <v>592</v>
+      </c>
+      <c r="C134" s="16" t="s">
+        <v>591</v>
+      </c>
+      <c r="D134" s="16" t="s">
+        <v>593</v>
+      </c>
+      <c r="E134" s="16" t="s">
+        <v>591</v>
+      </c>
+      <c r="F134" s="16" t="s">
+        <v>594</v>
+      </c>
+      <c r="G134" s="16"/>
+      <c r="H134" s="17"/>
+      <c r="I134" s="34" t="s">
+        <v>598</v>
+      </c>
+      <c r="J134" s="31"/>
+    </row>
+    <row r="135" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="20">
+        <f t="shared" si="1"/>
+        <v>133</v>
+      </c>
+      <c r="B135" s="28" t="s">
+        <v>592</v>
+      </c>
+      <c r="C135" s="16" t="s">
+        <v>591</v>
+      </c>
+      <c r="D135" s="16" t="s">
+        <v>595</v>
+      </c>
+      <c r="E135" s="16" t="s">
+        <v>591</v>
+      </c>
+      <c r="F135" s="16" t="s">
+        <v>596</v>
+      </c>
+      <c r="G135" s="14"/>
+      <c r="H135" s="15"/>
+      <c r="I135" s="14"/>
+      <c r="J135" s="30"/>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A136" s="9"/>
+      <c r="B136" s="18"/>
+      <c r="C136" s="10"/>
+      <c r="D136" s="11"/>
+      <c r="E136" s="12"/>
+      <c r="F136" s="13"/>
+      <c r="G136" s="12"/>
+      <c r="H136" s="13"/>
+      <c r="I136" s="13"/>
+      <c r="J136" s="13"/>
+    </row>
+    <row r="137" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A137" s="5"/>
+      <c r="B137" s="19"/>
+      <c r="C137" s="2"/>
+      <c r="D137" s="3"/>
+      <c r="E137" s="3"/>
+      <c r="F137" s="3"/>
+      <c r="G137" s="3"/>
+      <c r="H137" s="3"/>
+      <c r="I137" s="3"/>
+      <c r="J137" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H1:J1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="I134" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#15 Ze08-CH20 Sensor Added in Peripheral.
</commit_message>
<xml_diff>
--- a/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Client BOM tracker-pro-airbnb-v1.1.xlsx
+++ b/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Client BOM tracker-pro-airbnb-v1.1.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="599">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="600">
   <si>
     <t>#</t>
   </si>
@@ -1816,6 +1816,9 @@
   </si>
   <si>
     <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>ZE08-CH2O</t>
   </si>
 </sst>
 </file>
@@ -2185,9 +2188,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2208,6 +2208,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2497,7 +2500,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J137"/>
+  <dimension ref="A1:J138"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" style="6" bestFit="1" customWidth="1"/>
@@ -2520,9 +2523,9 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
@@ -2552,7 +2555,7 @@
       <c r="I2" s="7" t="s">
         <v>597</v>
       </c>
-      <c r="J2" s="29" t="s">
+      <c r="J2" s="28" t="s">
         <v>589</v>
       </c>
     </row>
@@ -2583,7 +2586,7 @@
         <v>529</v>
       </c>
       <c r="I3" s="14"/>
-      <c r="J3" s="30">
+      <c r="J3" s="29">
         <v>12</v>
       </c>
     </row>
@@ -2614,7 +2617,7 @@
         <v>530</v>
       </c>
       <c r="I4" s="16"/>
-      <c r="J4" s="31">
+      <c r="J4" s="30">
         <v>1</v>
       </c>
     </row>
@@ -2645,7 +2648,7 @@
         <v>531</v>
       </c>
       <c r="I5" s="14"/>
-      <c r="J5" s="30">
+      <c r="J5" s="29">
         <v>39</v>
       </c>
     </row>
@@ -2676,7 +2679,7 @@
         <v>532</v>
       </c>
       <c r="I6" s="16"/>
-      <c r="J6" s="31">
+      <c r="J6" s="30">
         <v>1</v>
       </c>
     </row>
@@ -2707,7 +2710,7 @@
         <v>533</v>
       </c>
       <c r="I7" s="14"/>
-      <c r="J7" s="30">
+      <c r="J7" s="29">
         <v>2</v>
       </c>
     </row>
@@ -2738,7 +2741,7 @@
         <v>534</v>
       </c>
       <c r="I8" s="16"/>
-      <c r="J8" s="31">
+      <c r="J8" s="30">
         <v>1</v>
       </c>
     </row>
@@ -2769,7 +2772,7 @@
         <v>535</v>
       </c>
       <c r="I9" s="14"/>
-      <c r="J9" s="30">
+      <c r="J9" s="29">
         <v>17</v>
       </c>
     </row>
@@ -2800,7 +2803,7 @@
         <v>536</v>
       </c>
       <c r="I10" s="16"/>
-      <c r="J10" s="31">
+      <c r="J10" s="30">
         <v>1</v>
       </c>
     </row>
@@ -2831,7 +2834,7 @@
         <v>537</v>
       </c>
       <c r="I11" s="14"/>
-      <c r="J11" s="30">
+      <c r="J11" s="29">
         <v>3</v>
       </c>
     </row>
@@ -2862,7 +2865,7 @@
         <v>538</v>
       </c>
       <c r="I12" s="16"/>
-      <c r="J12" s="31">
+      <c r="J12" s="30">
         <v>2</v>
       </c>
     </row>
@@ -2893,7 +2896,7 @@
         <v>539</v>
       </c>
       <c r="I13" s="14"/>
-      <c r="J13" s="30">
+      <c r="J13" s="29">
         <v>2</v>
       </c>
     </row>
@@ -2924,7 +2927,7 @@
         <v>529</v>
       </c>
       <c r="I14" s="16"/>
-      <c r="J14" s="31">
+      <c r="J14" s="30">
         <v>1</v>
       </c>
     </row>
@@ -2955,7 +2958,7 @@
         <v>540</v>
       </c>
       <c r="I15" s="14"/>
-      <c r="J15" s="30">
+      <c r="J15" s="29">
         <v>1</v>
       </c>
     </row>
@@ -2986,7 +2989,7 @@
         <v>541</v>
       </c>
       <c r="I16" s="16"/>
-      <c r="J16" s="31">
+      <c r="J16" s="30">
         <v>2</v>
       </c>
     </row>
@@ -3017,7 +3020,7 @@
         <v>533</v>
       </c>
       <c r="I17" s="14"/>
-      <c r="J17" s="30">
+      <c r="J17" s="29">
         <v>3</v>
       </c>
     </row>
@@ -3048,7 +3051,7 @@
         <v>542</v>
       </c>
       <c r="I18" s="16"/>
-      <c r="J18" s="31">
+      <c r="J18" s="30">
         <v>1</v>
       </c>
     </row>
@@ -3079,7 +3082,7 @@
         <v>531</v>
       </c>
       <c r="I19" s="14"/>
-      <c r="J19" s="30">
+      <c r="J19" s="29">
         <v>2</v>
       </c>
     </row>
@@ -3110,7 +3113,7 @@
         <v>543</v>
       </c>
       <c r="I20" s="16"/>
-      <c r="J20" s="31">
+      <c r="J20" s="30">
         <v>1</v>
       </c>
     </row>
@@ -3141,7 +3144,7 @@
         <v>544</v>
       </c>
       <c r="I21" s="14"/>
-      <c r="J21" s="30">
+      <c r="J21" s="29">
         <v>2</v>
       </c>
     </row>
@@ -3172,7 +3175,7 @@
         <v>545</v>
       </c>
       <c r="I22" s="16"/>
-      <c r="J22" s="31">
+      <c r="J22" s="30">
         <v>1</v>
       </c>
     </row>
@@ -3203,7 +3206,7 @@
         <v>533</v>
       </c>
       <c r="I23" s="14"/>
-      <c r="J23" s="30">
+      <c r="J23" s="29">
         <v>2</v>
       </c>
     </row>
@@ -3234,7 +3237,7 @@
         <v>529</v>
       </c>
       <c r="I24" s="16"/>
-      <c r="J24" s="31">
+      <c r="J24" s="30">
         <v>2</v>
       </c>
     </row>
@@ -3265,7 +3268,7 @@
         <v>546</v>
       </c>
       <c r="I25" s="14"/>
-      <c r="J25" s="30">
+      <c r="J25" s="29">
         <v>3</v>
       </c>
     </row>
@@ -3296,7 +3299,7 @@
         <v>547</v>
       </c>
       <c r="I26" s="16"/>
-      <c r="J26" s="31">
+      <c r="J26" s="30">
         <v>1</v>
       </c>
     </row>
@@ -3327,7 +3330,7 @@
         <v>548</v>
       </c>
       <c r="I27" s="14"/>
-      <c r="J27" s="30">
+      <c r="J27" s="29">
         <v>1</v>
       </c>
     </row>
@@ -3358,7 +3361,7 @@
         <v>531</v>
       </c>
       <c r="I28" s="16"/>
-      <c r="J28" s="31">
+      <c r="J28" s="30">
         <v>4</v>
       </c>
     </row>
@@ -3389,7 +3392,7 @@
         <v>537</v>
       </c>
       <c r="I29" s="14"/>
-      <c r="J29" s="30">
+      <c r="J29" s="29">
         <v>1</v>
       </c>
     </row>
@@ -3420,7 +3423,7 @@
         <v>549</v>
       </c>
       <c r="I30" s="16"/>
-      <c r="J30" s="31">
+      <c r="J30" s="30">
         <v>1</v>
       </c>
     </row>
@@ -3451,7 +3454,7 @@
         <v>531</v>
       </c>
       <c r="I31" s="14"/>
-      <c r="J31" s="30">
+      <c r="J31" s="29">
         <v>1</v>
       </c>
     </row>
@@ -3482,7 +3485,7 @@
         <v>529</v>
       </c>
       <c r="I32" s="16"/>
-      <c r="J32" s="31">
+      <c r="J32" s="30">
         <v>4</v>
       </c>
     </row>
@@ -3513,7 +3516,7 @@
         <v>591</v>
       </c>
       <c r="I33" s="14"/>
-      <c r="J33" s="30">
+      <c r="J33" s="29">
         <v>1</v>
       </c>
     </row>
@@ -3544,7 +3547,7 @@
         <v>550</v>
       </c>
       <c r="I34" s="23"/>
-      <c r="J34" s="32">
+      <c r="J34" s="31">
         <v>1</v>
       </c>
     </row>
@@ -3575,7 +3578,7 @@
         <v>591</v>
       </c>
       <c r="I35" s="14"/>
-      <c r="J35" s="30">
+      <c r="J35" s="29">
         <v>2</v>
       </c>
     </row>
@@ -3606,7 +3609,7 @@
         <v>591</v>
       </c>
       <c r="I36" s="14"/>
-      <c r="J36" s="31">
+      <c r="J36" s="30">
         <v>1</v>
       </c>
     </row>
@@ -3637,7 +3640,7 @@
         <v>591</v>
       </c>
       <c r="I37" s="14"/>
-      <c r="J37" s="30">
+      <c r="J37" s="29">
         <v>1</v>
       </c>
     </row>
@@ -3668,7 +3671,7 @@
         <v>591</v>
       </c>
       <c r="I38" s="14"/>
-      <c r="J38" s="31">
+      <c r="J38" s="30">
         <v>1</v>
       </c>
     </row>
@@ -3699,7 +3702,7 @@
         <v>591</v>
       </c>
       <c r="I39" s="14"/>
-      <c r="J39" s="30">
+      <c r="J39" s="29">
         <v>1</v>
       </c>
     </row>
@@ -3730,7 +3733,7 @@
         <v>591</v>
       </c>
       <c r="I40" s="14"/>
-      <c r="J40" s="31">
+      <c r="J40" s="30">
         <v>2</v>
       </c>
     </row>
@@ -3761,7 +3764,7 @@
         <v>591</v>
       </c>
       <c r="I41" s="14"/>
-      <c r="J41" s="30">
+      <c r="J41" s="29">
         <v>5</v>
       </c>
     </row>
@@ -3792,7 +3795,7 @@
         <v>591</v>
       </c>
       <c r="I42" s="14"/>
-      <c r="J42" s="31">
+      <c r="J42" s="30">
         <v>3</v>
       </c>
     </row>
@@ -3823,7 +3826,7 @@
         <v>591</v>
       </c>
       <c r="I43" s="14"/>
-      <c r="J43" s="30">
+      <c r="J43" s="29">
         <v>2</v>
       </c>
     </row>
@@ -3854,7 +3857,7 @@
         <v>551</v>
       </c>
       <c r="I44" s="16"/>
-      <c r="J44" s="31">
+      <c r="J44" s="30">
         <v>7</v>
       </c>
     </row>
@@ -3885,7 +3888,7 @@
         <v>591</v>
       </c>
       <c r="I45" s="14"/>
-      <c r="J45" s="30">
+      <c r="J45" s="29">
         <v>1</v>
       </c>
     </row>
@@ -3916,7 +3919,7 @@
         <v>591</v>
       </c>
       <c r="I46" s="14"/>
-      <c r="J46" s="31">
+      <c r="J46" s="30">
         <v>1</v>
       </c>
     </row>
@@ -3947,7 +3950,7 @@
         <v>591</v>
       </c>
       <c r="I47" s="14"/>
-      <c r="J47" s="30">
+      <c r="J47" s="29">
         <v>1</v>
       </c>
     </row>
@@ -3978,7 +3981,7 @@
         <v>591</v>
       </c>
       <c r="I48" s="14"/>
-      <c r="J48" s="31">
+      <c r="J48" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4009,7 +4012,7 @@
         <v>591</v>
       </c>
       <c r="I49" s="14"/>
-      <c r="J49" s="30">
+      <c r="J49" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4040,7 +4043,7 @@
         <v>591</v>
       </c>
       <c r="I50" s="14"/>
-      <c r="J50" s="31">
+      <c r="J50" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4071,7 +4074,7 @@
         <v>591</v>
       </c>
       <c r="I51" s="14"/>
-      <c r="J51" s="30">
+      <c r="J51" s="29">
         <v>3</v>
       </c>
     </row>
@@ -4100,7 +4103,7 @@
         <v>591</v>
       </c>
       <c r="I52" s="14"/>
-      <c r="J52" s="31">
+      <c r="J52" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4131,7 +4134,7 @@
         <v>591</v>
       </c>
       <c r="I53" s="14"/>
-      <c r="J53" s="30">
+      <c r="J53" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4162,7 +4165,7 @@
         <v>591</v>
       </c>
       <c r="I54" s="14"/>
-      <c r="J54" s="31">
+      <c r="J54" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4193,7 +4196,7 @@
         <v>552</v>
       </c>
       <c r="I55" s="14"/>
-      <c r="J55" s="30">
+      <c r="J55" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4224,7 +4227,7 @@
         <v>553</v>
       </c>
       <c r="I56" s="16"/>
-      <c r="J56" s="31">
+      <c r="J56" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4255,7 +4258,7 @@
         <v>554</v>
       </c>
       <c r="I57" s="14"/>
-      <c r="J57" s="30">
+      <c r="J57" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4286,7 +4289,7 @@
         <v>555</v>
       </c>
       <c r="I58" s="16"/>
-      <c r="J58" s="31">
+      <c r="J58" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4317,7 +4320,7 @@
         <v>591</v>
       </c>
       <c r="I59" s="14"/>
-      <c r="J59" s="30">
+      <c r="J59" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4348,7 +4351,7 @@
         <v>591</v>
       </c>
       <c r="I60" s="14"/>
-      <c r="J60" s="31">
+      <c r="J60" s="30">
         <v>2</v>
       </c>
     </row>
@@ -4379,7 +4382,7 @@
         <v>591</v>
       </c>
       <c r="I61" s="14"/>
-      <c r="J61" s="30">
+      <c r="J61" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4410,7 +4413,7 @@
         <v>591</v>
       </c>
       <c r="I62" s="14"/>
-      <c r="J62" s="31">
+      <c r="J62" s="30">
         <v>5</v>
       </c>
     </row>
@@ -4437,7 +4440,7 @@
         <v>591</v>
       </c>
       <c r="I63" s="25"/>
-      <c r="J63" s="33">
+      <c r="J63" s="32">
         <v>21</v>
       </c>
     </row>
@@ -4468,7 +4471,7 @@
         <v>550</v>
       </c>
       <c r="I64" s="23"/>
-      <c r="J64" s="32">
+      <c r="J64" s="31">
         <v>1</v>
       </c>
     </row>
@@ -4499,7 +4502,7 @@
         <v>591</v>
       </c>
       <c r="I65" s="14"/>
-      <c r="J65" s="30">
+      <c r="J65" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4530,7 +4533,7 @@
         <v>591</v>
       </c>
       <c r="I66" s="14"/>
-      <c r="J66" s="31">
+      <c r="J66" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4561,7 +4564,7 @@
         <v>591</v>
       </c>
       <c r="I67" s="14"/>
-      <c r="J67" s="30">
+      <c r="J67" s="29">
         <v>2</v>
       </c>
     </row>
@@ -4592,7 +4595,7 @@
         <v>591</v>
       </c>
       <c r="I68" s="14"/>
-      <c r="J68" s="31">
+      <c r="J68" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4623,7 +4626,7 @@
         <v>591</v>
       </c>
       <c r="I69" s="14"/>
-      <c r="J69" s="30">
+      <c r="J69" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4654,7 +4657,7 @@
         <v>556</v>
       </c>
       <c r="I70" s="16"/>
-      <c r="J70" s="31">
+      <c r="J70" s="30">
         <v>4</v>
       </c>
     </row>
@@ -4685,7 +4688,7 @@
         <v>557</v>
       </c>
       <c r="I71" s="14"/>
-      <c r="J71" s="30">
+      <c r="J71" s="29">
         <v>2</v>
       </c>
     </row>
@@ -4716,7 +4719,7 @@
         <v>558</v>
       </c>
       <c r="I72" s="16"/>
-      <c r="J72" s="31">
+      <c r="J72" s="30">
         <v>20</v>
       </c>
     </row>
@@ -4747,7 +4750,7 @@
         <v>559</v>
       </c>
       <c r="I73" s="14"/>
-      <c r="J73" s="30">
+      <c r="J73" s="29">
         <v>6</v>
       </c>
     </row>
@@ -4778,7 +4781,7 @@
         <v>560</v>
       </c>
       <c r="I74" s="16"/>
-      <c r="J74" s="31">
+      <c r="J74" s="30">
         <v>2</v>
       </c>
     </row>
@@ -4809,7 +4812,7 @@
         <v>561</v>
       </c>
       <c r="I75" s="14"/>
-      <c r="J75" s="30">
+      <c r="J75" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4840,7 +4843,7 @@
         <v>562</v>
       </c>
       <c r="I76" s="16"/>
-      <c r="J76" s="31">
+      <c r="J76" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4871,7 +4874,7 @@
         <v>563</v>
       </c>
       <c r="I77" s="14"/>
-      <c r="J77" s="30">
+      <c r="J77" s="29">
         <v>1</v>
       </c>
     </row>
@@ -4902,7 +4905,7 @@
         <v>564</v>
       </c>
       <c r="I78" s="16"/>
-      <c r="J78" s="31">
+      <c r="J78" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4933,7 +4936,7 @@
         <v>550</v>
       </c>
       <c r="I79" s="25"/>
-      <c r="J79" s="33">
+      <c r="J79" s="32">
         <v>1</v>
       </c>
     </row>
@@ -4964,7 +4967,7 @@
         <v>565</v>
       </c>
       <c r="I80" s="16"/>
-      <c r="J80" s="31">
+      <c r="J80" s="30">
         <v>1</v>
       </c>
     </row>
@@ -4995,7 +4998,7 @@
         <v>566</v>
       </c>
       <c r="I81" s="14"/>
-      <c r="J81" s="30">
+      <c r="J81" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5026,7 +5029,7 @@
         <v>567</v>
       </c>
       <c r="I82" s="16"/>
-      <c r="J82" s="31">
+      <c r="J82" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5057,7 +5060,7 @@
         <v>568</v>
       </c>
       <c r="I83" s="14"/>
-      <c r="J83" s="30">
+      <c r="J83" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5088,7 +5091,7 @@
         <v>569</v>
       </c>
       <c r="I84" s="16"/>
-      <c r="J84" s="31">
+      <c r="J84" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5119,7 +5122,7 @@
         <v>558</v>
       </c>
       <c r="I85" s="14"/>
-      <c r="J85" s="30">
+      <c r="J85" s="29">
         <v>6</v>
       </c>
     </row>
@@ -5150,7 +5153,7 @@
         <v>570</v>
       </c>
       <c r="I86" s="16"/>
-      <c r="J86" s="31">
+      <c r="J86" s="30">
         <v>3</v>
       </c>
     </row>
@@ -5181,7 +5184,7 @@
         <v>571</v>
       </c>
       <c r="I87" s="14"/>
-      <c r="J87" s="30">
+      <c r="J87" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5212,7 +5215,7 @@
         <v>572</v>
       </c>
       <c r="I88" s="16"/>
-      <c r="J88" s="31">
+      <c r="J88" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5243,7 +5246,7 @@
         <v>573</v>
       </c>
       <c r="I89" s="14"/>
-      <c r="J89" s="30">
+      <c r="J89" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5274,7 +5277,7 @@
         <v>574</v>
       </c>
       <c r="I90" s="16"/>
-      <c r="J90" s="31">
+      <c r="J90" s="30">
         <v>2</v>
       </c>
     </row>
@@ -5305,7 +5308,7 @@
         <v>575</v>
       </c>
       <c r="I91" s="14"/>
-      <c r="J91" s="30">
+      <c r="J91" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5336,7 +5339,7 @@
         <v>576</v>
       </c>
       <c r="I92" s="16"/>
-      <c r="J92" s="31">
+      <c r="J92" s="30">
         <v>4</v>
       </c>
     </row>
@@ -5367,7 +5370,7 @@
         <v>577</v>
       </c>
       <c r="I93" s="14"/>
-      <c r="J93" s="30">
+      <c r="J93" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5398,7 +5401,7 @@
         <v>578</v>
       </c>
       <c r="I94" s="16"/>
-      <c r="J94" s="31">
+      <c r="J94" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5429,7 +5432,7 @@
         <v>579</v>
       </c>
       <c r="I95" s="14"/>
-      <c r="J95" s="30">
+      <c r="J95" s="29">
         <v>4</v>
       </c>
     </row>
@@ -5460,7 +5463,7 @@
         <v>580</v>
       </c>
       <c r="I96" s="16"/>
-      <c r="J96" s="31">
+      <c r="J96" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5491,7 +5494,7 @@
         <v>581</v>
       </c>
       <c r="I97" s="14"/>
-      <c r="J97" s="30">
+      <c r="J97" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5522,7 +5525,7 @@
         <v>582</v>
       </c>
       <c r="I98" s="16"/>
-      <c r="J98" s="31">
+      <c r="J98" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5553,7 +5556,7 @@
         <v>583</v>
       </c>
       <c r="I99" s="14"/>
-      <c r="J99" s="30">
+      <c r="J99" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5584,7 +5587,7 @@
         <v>558</v>
       </c>
       <c r="I100" s="16"/>
-      <c r="J100" s="31">
+      <c r="J100" s="30">
         <v>3</v>
       </c>
     </row>
@@ -5613,7 +5616,7 @@
         <v>591</v>
       </c>
       <c r="I101" s="25"/>
-      <c r="J101" s="33">
+      <c r="J101" s="32">
         <v>4</v>
       </c>
     </row>
@@ -5642,7 +5645,7 @@
         <v>591</v>
       </c>
       <c r="I102" s="25"/>
-      <c r="J102" s="32">
+      <c r="J102" s="31">
         <v>2</v>
       </c>
     </row>
@@ -5673,7 +5676,7 @@
         <v>591</v>
       </c>
       <c r="I103" s="14"/>
-      <c r="J103" s="30">
+      <c r="J103" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5704,7 +5707,7 @@
         <v>591</v>
       </c>
       <c r="I104" s="14"/>
-      <c r="J104" s="31">
+      <c r="J104" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5735,7 +5738,7 @@
         <v>591</v>
       </c>
       <c r="I105" s="14"/>
-      <c r="J105" s="30">
+      <c r="J105" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5766,7 +5769,7 @@
         <v>591</v>
       </c>
       <c r="I106" s="14"/>
-      <c r="J106" s="31">
+      <c r="J106" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5797,7 +5800,7 @@
         <v>591</v>
       </c>
       <c r="I107" s="14"/>
-      <c r="J107" s="30">
+      <c r="J107" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5828,7 +5831,7 @@
         <v>591</v>
       </c>
       <c r="I108" s="14"/>
-      <c r="J108" s="31">
+      <c r="J108" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5859,7 +5862,7 @@
         <v>591</v>
       </c>
       <c r="I109" s="14"/>
-      <c r="J109" s="30">
+      <c r="J109" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5890,7 +5893,7 @@
         <v>591</v>
       </c>
       <c r="I110" s="14"/>
-      <c r="J110" s="31">
+      <c r="J110" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5921,7 +5924,7 @@
         <v>591</v>
       </c>
       <c r="I111" s="14"/>
-      <c r="J111" s="30">
+      <c r="J111" s="29">
         <v>1</v>
       </c>
     </row>
@@ -5952,7 +5955,7 @@
         <v>591</v>
       </c>
       <c r="I112" s="14"/>
-      <c r="J112" s="31">
+      <c r="J112" s="30">
         <v>1</v>
       </c>
     </row>
@@ -5983,7 +5986,7 @@
         <v>591</v>
       </c>
       <c r="I113" s="14"/>
-      <c r="J113" s="30">
+      <c r="J113" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6014,7 +6017,7 @@
         <v>591</v>
       </c>
       <c r="I114" s="14"/>
-      <c r="J114" s="31">
+      <c r="J114" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6045,7 +6048,7 @@
         <v>591</v>
       </c>
       <c r="I115" s="14"/>
-      <c r="J115" s="30">
+      <c r="J115" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6076,7 +6079,7 @@
         <v>591</v>
       </c>
       <c r="I116" s="14"/>
-      <c r="J116" s="31">
+      <c r="J116" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6107,7 +6110,7 @@
         <v>591</v>
       </c>
       <c r="I117" s="14"/>
-      <c r="J117" s="30">
+      <c r="J117" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6138,7 +6141,7 @@
         <v>591</v>
       </c>
       <c r="I118" s="14"/>
-      <c r="J118" s="31">
+      <c r="J118" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6169,7 +6172,7 @@
         <v>591</v>
       </c>
       <c r="I119" s="14"/>
-      <c r="J119" s="30">
+      <c r="J119" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6200,7 +6203,7 @@
         <v>591</v>
       </c>
       <c r="I120" s="14"/>
-      <c r="J120" s="31">
+      <c r="J120" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6231,7 +6234,7 @@
         <v>591</v>
       </c>
       <c r="I121" s="14"/>
-      <c r="J121" s="30">
+      <c r="J121" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6262,7 +6265,7 @@
         <v>591</v>
       </c>
       <c r="I122" s="14"/>
-      <c r="J122" s="31">
+      <c r="J122" s="30">
         <v>4</v>
       </c>
     </row>
@@ -6293,7 +6296,7 @@
         <v>591</v>
       </c>
       <c r="I123" s="14"/>
-      <c r="J123" s="30">
+      <c r="J123" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6324,7 +6327,7 @@
         <v>591</v>
       </c>
       <c r="I124" s="14"/>
-      <c r="J124" s="31">
+      <c r="J124" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6355,7 +6358,7 @@
         <v>591</v>
       </c>
       <c r="I125" s="14"/>
-      <c r="J125" s="30">
+      <c r="J125" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6386,7 +6389,7 @@
         <v>591</v>
       </c>
       <c r="I126" s="14"/>
-      <c r="J126" s="31">
+      <c r="J126" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6417,7 +6420,7 @@
         <v>591</v>
       </c>
       <c r="I127" s="14"/>
-      <c r="J127" s="30">
+      <c r="J127" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6448,7 +6451,7 @@
         <v>591</v>
       </c>
       <c r="I128" s="14"/>
-      <c r="J128" s="31">
+      <c r="J128" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6479,7 +6482,7 @@
         <v>584</v>
       </c>
       <c r="I129" s="14"/>
-      <c r="J129" s="30">
+      <c r="J129" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6510,7 +6513,7 @@
         <v>585</v>
       </c>
       <c r="I130" s="16"/>
-      <c r="J130" s="31">
+      <c r="J130" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6541,7 +6544,7 @@
         <v>586</v>
       </c>
       <c r="I131" s="14"/>
-      <c r="J131" s="30">
+      <c r="J131" s="29">
         <v>1</v>
       </c>
     </row>
@@ -6572,7 +6575,7 @@
         <v>587</v>
       </c>
       <c r="I132" s="16"/>
-      <c r="J132" s="31">
+      <c r="J132" s="30">
         <v>1</v>
       </c>
     </row>
@@ -6603,16 +6606,16 @@
         <v>588</v>
       </c>
       <c r="I133" s="14"/>
-      <c r="J133" s="30">
+      <c r="J133" s="29">
         <v>1</v>
       </c>
     </row>
     <row r="134" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="20">
-        <f t="shared" ref="A134:A135" si="1">ROW(A134) - ROW($A$2)</f>
+        <f t="shared" ref="A134:A136" si="1">ROW(A134) - ROW($A$2)</f>
         <v>132</v>
       </c>
-      <c r="B134" s="28" t="s">
+      <c r="B134" s="27" t="s">
         <v>592</v>
       </c>
       <c r="C134" s="16" t="s">
@@ -6629,17 +6632,17 @@
       </c>
       <c r="G134" s="16"/>
       <c r="H134" s="17"/>
-      <c r="I134" s="34" t="s">
+      <c r="I134" s="33" t="s">
         <v>598</v>
       </c>
-      <c r="J134" s="31"/>
+      <c r="J134" s="30"/>
     </row>
     <row r="135" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="20">
         <f t="shared" si="1"/>
         <v>133</v>
       </c>
-      <c r="B135" s="28" t="s">
+      <c r="B135" s="27" t="s">
         <v>592</v>
       </c>
       <c r="C135" s="16" t="s">
@@ -6657,31 +6660,56 @@
       <c r="G135" s="14"/>
       <c r="H135" s="15"/>
       <c r="I135" s="14"/>
-      <c r="J135" s="30"/>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A136" s="9"/>
-      <c r="B136" s="18"/>
-      <c r="C136" s="10"/>
-      <c r="D136" s="11"/>
-      <c r="E136" s="12"/>
-      <c r="F136" s="13"/>
-      <c r="G136" s="12"/>
-      <c r="H136" s="13"/>
-      <c r="I136" s="13"/>
-      <c r="J136" s="13"/>
-    </row>
-    <row r="137" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="5"/>
-      <c r="B137" s="19"/>
-      <c r="C137" s="2"/>
-      <c r="D137" s="3"/>
-      <c r="E137" s="3"/>
-      <c r="F137" s="3"/>
-      <c r="G137" s="3"/>
-      <c r="H137" s="3"/>
-      <c r="I137" s="3"/>
-      <c r="J137" s="3"/>
+      <c r="J135" s="29"/>
+    </row>
+    <row r="136" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="20">
+        <f t="shared" si="1"/>
+        <v>134</v>
+      </c>
+      <c r="B136" s="27" t="s">
+        <v>592</v>
+      </c>
+      <c r="C136" s="16" t="s">
+        <v>591</v>
+      </c>
+      <c r="D136" s="16" t="s">
+        <v>595</v>
+      </c>
+      <c r="E136" s="16" t="s">
+        <v>591</v>
+      </c>
+      <c r="F136" s="16" t="s">
+        <v>599</v>
+      </c>
+      <c r="G136" s="14"/>
+      <c r="H136" s="15"/>
+      <c r="I136" s="14"/>
+      <c r="J136" s="29"/>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A137" s="9"/>
+      <c r="B137" s="18"/>
+      <c r="C137" s="10"/>
+      <c r="D137" s="11"/>
+      <c r="E137" s="12"/>
+      <c r="F137" s="13"/>
+      <c r="G137" s="12"/>
+      <c r="H137" s="13"/>
+      <c r="I137" s="13"/>
+      <c r="J137" s="13"/>
+    </row>
+    <row r="138" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="5"/>
+      <c r="B138" s="19"/>
+      <c r="C138" s="2"/>
+      <c r="D138" s="3"/>
+      <c r="E138" s="3"/>
+      <c r="F138" s="3"/>
+      <c r="G138" s="3"/>
+      <c r="H138" s="3"/>
+      <c r="I138" s="3"/>
+      <c r="J138" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>